<commit_message>
Current working, need fixing on battery mode and list mode to work properly
</commit_message>
<xml_diff>
--- a/CAN_Commands_Database.xlsx
+++ b/CAN_Commands_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FinalProject_KMUTNB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{889E27D8-F600-4F5F-AC79-DCE1F82BAC6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{206C4DE4-DD57-4091-B20D-D7261E0612D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1500" yWindow="1500" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Phoenix_TRIO_HP" sheetId="1" r:id="rId1"/>
@@ -2686,10 +2686,11 @@
   <dimension ref="A1:G47"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="49.5546875" customWidth="1"/>
-    <col min="3" max="3" width="50.88671875" customWidth="1"/>
-    <col min="4" max="4" width="70" customWidth="1"/>
-    <col min="5" max="5" width="91.44140625" customWidth="1"/>
+    <col min="1" max="1" width="22.5546875" customWidth="1"/>
+    <col min="2" max="2" width="3.33203125" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" customWidth="1"/>
+    <col min="4" max="4" width="22.33203125" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>